<commit_message>
Refactor caminhos_pastas function to improve path handling and readability; add new e_viab and r_cef_empreend functions for viability data processing; update Template-DFC.xlsx.
</commit_message>
<xml_diff>
--- a/templates/Template-DFC.xlsx
+++ b/templates/Template-DFC.xlsx
@@ -1,20 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="198" documentId="8_{482EB0F2-8EC4-40C5-8B55-F33B1732A6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55FC653C-C221-486A-A344-A744A9E94705}"/>
+  <xr:revisionPtr revIDLastSave="199" documentId="8_{482EB0F2-8EC4-40C5-8B55-F33B1732A6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D45E27F8-55D0-4F81-B847-B7A8454F993A}"/>
   <bookViews>
-    <workbookView xWindow="-14400" yWindow="-1185" windowWidth="14400" windowHeight="15600" xr2:uid="{E8652140-B299-493A-AAA8-27682F0F7EF9}"/>
+    <workbookView xWindow="-20370" yWindow="1245" windowWidth="15375" windowHeight="7215" firstSheet="1" activeTab="3" xr2:uid="{E8652140-B299-493A-AAA8-27682F0F7EF9}"/>
   </bookViews>
   <sheets>
     <sheet name="Por empresa" sheetId="1" r:id="rId1"/>
     <sheet name="Por empreendimento" sheetId="2" r:id="rId2"/>
+    <sheet name="DFC_Direto" sheetId="3" r:id="rId3"/>
+    <sheet name="Notas_e_Instruções" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="137">
   <si>
     <t>Código</t>
   </si>
@@ -175,13 +177,286 @@
   </si>
   <si>
     <t>Impostos e outras despesas legais</t>
+  </si>
+  <si>
+    <t>Caixa e Equivalentes no Fim do Período</t>
+  </si>
+  <si>
+    <t>4.03</t>
+  </si>
+  <si>
+    <t>Caixa e Equivalentes no Início do Período</t>
+  </si>
+  <si>
+    <t>4.02</t>
+  </si>
+  <si>
+    <t>Variação Líquida de Caixa no Período</t>
+  </si>
+  <si>
+    <t>4.01</t>
+  </si>
+  <si>
+    <t>Caixa Líquido das Atividades de Financiamento</t>
+  </si>
+  <si>
+    <t>3.98</t>
+  </si>
+  <si>
+    <t>Outros Pagamentos de Financiamento</t>
+  </si>
+  <si>
+    <t>3.08</t>
+  </si>
+  <si>
+    <t>Distribuição de Dividendos / JCP</t>
+  </si>
+  <si>
+    <t>3.07</t>
+  </si>
+  <si>
+    <t>Pagamento de Juros</t>
+  </si>
+  <si>
+    <t>3.06</t>
+  </si>
+  <si>
+    <t>Amortização de Empréstimos / Financiamentos</t>
+  </si>
+  <si>
+    <t>3.05</t>
+  </si>
+  <si>
+    <t>Outros Financiamentos (Entradas)</t>
+  </si>
+  <si>
+    <t>3.04</t>
+  </si>
+  <si>
+    <t>Aporte de Capital dos Sócios</t>
+  </si>
+  <si>
+    <t>3.03</t>
+  </si>
+  <si>
+    <t>Emissão de Debêntures</t>
+  </si>
+  <si>
+    <t>3.02</t>
+  </si>
+  <si>
+    <t>Captação de Empréstimos / Financiamentos Bancários</t>
+  </si>
+  <si>
+    <t>3.01</t>
+  </si>
+  <si>
+    <t>Caixa Líquido das Atividades de Investimento</t>
+  </si>
+  <si>
+    <t>2.98</t>
+  </si>
+  <si>
+    <t>Outros Investimentos</t>
+  </si>
+  <si>
+    <t>2.07</t>
+  </si>
+  <si>
+    <t>Investimento em Participações / SPEs</t>
+  </si>
+  <si>
+    <t>2.06</t>
+  </si>
+  <si>
+    <t>Aquisição de Equipamentos</t>
+  </si>
+  <si>
+    <t>2.05</t>
+  </si>
+  <si>
+    <t>Investimento em Construção e Obras em Andamento</t>
+  </si>
+  <si>
+    <t>2.04</t>
+  </si>
+  <si>
+    <t>Aquisição de Terrenos</t>
+  </si>
+  <si>
+    <t>2.03</t>
+  </si>
+  <si>
+    <t>Recebimentos de Juros sobre Aplicações</t>
+  </si>
+  <si>
+    <t>2.02</t>
+  </si>
+  <si>
+    <t>Venda de Ativos Imobilizados/Terrenos</t>
+  </si>
+  <si>
+    <t>2.01</t>
+  </si>
+  <si>
+    <t>Caixa Líquido das Atividades Operacionais</t>
+  </si>
+  <si>
+    <t>1.98</t>
+  </si>
+  <si>
+    <t>Outras Despesas Operacionais</t>
+  </si>
+  <si>
+    <t>1.11</t>
+  </si>
+  <si>
+    <t>Impostos e Contribuições sobre Receita</t>
+  </si>
+  <si>
+    <t>1.10</t>
+  </si>
+  <si>
+    <t>Despesas Administrativas Gerais</t>
+  </si>
+  <si>
+    <t>1.09</t>
+  </si>
+  <si>
+    <t>Despesas Comerciais e de Marketing</t>
+  </si>
+  <si>
+    <t>1.08</t>
+  </si>
+  <si>
+    <t>Pagamentos de Salários e Encargos</t>
+  </si>
+  <si>
+    <t>1.07</t>
+  </si>
+  <si>
+    <t>Pagamentos a Empreiteiros/Subempreiteiros</t>
+  </si>
+  <si>
+    <t>1.06</t>
+  </si>
+  <si>
+    <t>Pagamentos a Fornecedores (Materiais de Construção)</t>
+  </si>
+  <si>
+    <t>1.05</t>
+  </si>
+  <si>
+    <t>Subtotal Entradas Operacionais</t>
+  </si>
+  <si>
+    <t>1.99</t>
+  </si>
+  <si>
+    <t>Outras Receitas Operacionais</t>
+  </si>
+  <si>
+    <t>1.04</t>
+  </si>
+  <si>
+    <t>Recebimentos de Serviços (Taxas de Administração / Corretagem)</t>
+  </si>
+  <si>
+    <t>1.03</t>
+  </si>
+  <si>
+    <t>Recebimentos de Aluguéis</t>
+  </si>
+  <si>
+    <t>1.02</t>
+  </si>
+  <si>
+    <t>Recebimentos de Vendas de Unidades Imobiliárias</t>
+  </si>
+  <si>
+    <t>1.01</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Dez</t>
+  </si>
+  <si>
+    <t>Nov</t>
+  </si>
+  <si>
+    <t>Out</t>
+  </si>
+  <si>
+    <t>Set</t>
+  </si>
+  <si>
+    <t>Ago</t>
+  </si>
+  <si>
+    <t>Jul</t>
+  </si>
+  <si>
+    <t>Jun</t>
+  </si>
+  <si>
+    <t>Mai</t>
+  </si>
+  <si>
+    <t>Abr</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Fev</t>
+  </si>
+  <si>
+    <t>Jan</t>
+  </si>
+  <si>
+    <t>10. Proteja células de fórmulas para evitar alterações não intencionais.</t>
+  </si>
+  <si>
+    <t>9. Ajuste o mapeamento de contas conforme o plano de contas interno da Ampla.</t>
+  </si>
+  <si>
+    <t>8. Utilize referências absolutas nas fórmulas para manter a consistência ao copiar para novos períodos.</t>
+  </si>
+  <si>
+    <t>7. A variação líquida de caixa (4.01) deve ser a soma dos fluxos líquidos das três atividades.</t>
+  </si>
+  <si>
+    <t>6. Utilize as linhas de subtotal (1.99, 2.98, 3.98) para calcular automaticamente os fluxos líquidos por atividade.</t>
+  </si>
+  <si>
+    <t>5. Registre impostos sobre receita quando da saída de caixa, não pelo fato gerador contábil.</t>
+  </si>
+  <si>
+    <t>4. Detalhe pagamentos a fornecedores por grandes classes de custo (materiais, empreiteiros, etc.).</t>
+  </si>
+  <si>
+    <t>3. Agrupe os recebimentos de clientes por tipo de contrato (vendas, aluguéis, serviços).</t>
+  </si>
+  <si>
+    <t>2. Lance as entradas brutas de caixa separadamente das saídas para cada categoria.</t>
+  </si>
+  <si>
+    <t>1. Utilize apenas valores relacionados a movimentações de caixa efetivas (exclua receitas e despesas a prazo).</t>
+  </si>
+  <si>
+    <t>Orientações para preenchimento da Demonstração do Fluxo de Caixa (Método Direto):</t>
+  </si>
+  <si>
+    <t>Instruções</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -200,6 +475,14 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -243,7 +526,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -251,11 +534,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -296,6 +594,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1109,6 +1410,397 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DE0B94E-0419-42F5-8555-F770A44E2D08}">
+  <dimension ref="A1:O34"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="J1" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="K1" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="L1" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="M1" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="N1" s="15" t="s">
+        <v>113</v>
+      </c>
+      <c r="O1" s="15" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B5" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>101</v>
+      </c>
+      <c r="B7" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B8" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B11" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>91</v>
+      </c>
+      <c r="B12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>89</v>
+      </c>
+      <c r="B13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>85</v>
+      </c>
+      <c r="B15" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B16" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>79</v>
+      </c>
+      <c r="B18" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>77</v>
+      </c>
+      <c r="B19" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>75</v>
+      </c>
+      <c r="B20" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>73</v>
+      </c>
+      <c r="B21" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>71</v>
+      </c>
+      <c r="B22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>67</v>
+      </c>
+      <c r="B24" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>65</v>
+      </c>
+      <c r="B25" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>59</v>
+      </c>
+      <c r="B28" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>53</v>
+      </c>
+      <c r="B31" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>51</v>
+      </c>
+      <c r="B32" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>49</v>
+      </c>
+      <c r="B33" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>47</v>
+      </c>
+      <c r="B34" t="s">
+        <v>46</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EA864A3-80F6-45EA-B46F-4714BF885D6B}">
+  <dimension ref="A1:A12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="15" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>125</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
@@ -1305,15 +1997,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
@@ -1322,6 +2005,15 @@
     <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1344,14 +2036,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7BFC80B-7A55-4801-9844-CCCBA392669F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7E4AD77-7BCF-4163-8EFB-17D24A162300}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -1360,4 +2044,12 @@
     <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7BFC80B-7A55-4801-9844-CCCBA392669F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add e_extratos and e_extratos_mapa functions for extracting and mapping bank statement data; update NAMESPACE and documentation; replace outdated data files.
</commit_message>
<xml_diff>
--- a/templates/Template-DFC.xlsx
+++ b/templates/Template-DFC.xlsx
@@ -1,24 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="199" documentId="8_{482EB0F2-8EC4-40C5-8B55-F33B1732A6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D45E27F8-55D0-4F81-B847-B7A8454F993A}"/>
+  <xr:revisionPtr revIDLastSave="400" documentId="8_{482EB0F2-8EC4-40C5-8B55-F33B1732A6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56DE95E9-BB3E-41E9-BF20-7F01584FABD5}"/>
   <bookViews>
-    <workbookView xWindow="-20370" yWindow="1245" windowWidth="15375" windowHeight="7215" firstSheet="1" activeTab="3" xr2:uid="{E8652140-B299-493A-AAA8-27682F0F7EF9}"/>
+    <workbookView xWindow="-43200" yWindow="4245" windowWidth="14400" windowHeight="7800" activeTab="2" xr2:uid="{E8652140-B299-493A-AAA8-27682F0F7EF9}"/>
   </bookViews>
   <sheets>
-    <sheet name="Por empresa" sheetId="1" r:id="rId1"/>
-    <sheet name="Por empreendimento" sheetId="2" r:id="rId2"/>
-    <sheet name="DFC_Direto" sheetId="3" r:id="rId3"/>
-    <sheet name="Notas_e_Instruções" sheetId="4" r:id="rId4"/>
+    <sheet name="DFC" sheetId="1" r:id="rId1"/>
+    <sheet name="Mapeamento" sheetId="5" r:id="rId2"/>
+    <sheet name="Configurações" sheetId="6" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <externalReferences>
+    <externalReference r:id="rId4"/>
+  </externalReferences>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,8 +40,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="58">
   <si>
     <t>Código</t>
   </si>
@@ -179,284 +203,47 @@
     <t>Impostos e outras despesas legais</t>
   </si>
   <si>
-    <t>Caixa e Equivalentes no Fim do Período</t>
-  </si>
-  <si>
-    <t>4.03</t>
-  </si>
-  <si>
-    <t>Caixa e Equivalentes no Início do Período</t>
-  </si>
-  <si>
-    <t>4.02</t>
-  </si>
-  <si>
-    <t>Variação Líquida de Caixa no Período</t>
-  </si>
-  <si>
-    <t>4.01</t>
-  </si>
-  <si>
-    <t>Caixa Líquido das Atividades de Financiamento</t>
-  </si>
-  <si>
-    <t>3.98</t>
-  </si>
-  <si>
-    <t>Outros Pagamentos de Financiamento</t>
-  </si>
-  <si>
-    <t>3.08</t>
-  </si>
-  <si>
-    <t>Distribuição de Dividendos / JCP</t>
-  </si>
-  <si>
-    <t>3.07</t>
-  </si>
-  <si>
-    <t>Pagamento de Juros</t>
-  </si>
-  <si>
-    <t>3.06</t>
-  </si>
-  <si>
-    <t>Amortização de Empréstimos / Financiamentos</t>
-  </si>
-  <si>
-    <t>3.05</t>
-  </si>
-  <si>
-    <t>Outros Financiamentos (Entradas)</t>
-  </si>
-  <si>
-    <t>3.04</t>
-  </si>
-  <si>
-    <t>Aporte de Capital dos Sócios</t>
-  </si>
-  <si>
-    <t>3.03</t>
-  </si>
-  <si>
-    <t>Emissão de Debêntures</t>
-  </si>
-  <si>
-    <t>3.02</t>
-  </si>
-  <si>
-    <t>Captação de Empréstimos / Financiamentos Bancários</t>
-  </si>
-  <si>
-    <t>3.01</t>
-  </si>
-  <si>
-    <t>Caixa Líquido das Atividades de Investimento</t>
-  </si>
-  <si>
-    <t>2.98</t>
-  </si>
-  <si>
-    <t>Outros Investimentos</t>
-  </si>
-  <si>
-    <t>2.07</t>
-  </si>
-  <si>
-    <t>Investimento em Participações / SPEs</t>
-  </si>
-  <si>
-    <t>2.06</t>
-  </si>
-  <si>
-    <t>Aquisição de Equipamentos</t>
-  </si>
-  <si>
-    <t>2.05</t>
-  </si>
-  <si>
-    <t>Investimento em Construção e Obras em Andamento</t>
-  </si>
-  <si>
-    <t>2.04</t>
-  </si>
-  <si>
-    <t>Aquisição de Terrenos</t>
-  </si>
-  <si>
-    <t>2.03</t>
-  </si>
-  <si>
-    <t>Recebimentos de Juros sobre Aplicações</t>
-  </si>
-  <si>
-    <t>2.02</t>
-  </si>
-  <si>
-    <t>Venda de Ativos Imobilizados/Terrenos</t>
-  </si>
-  <si>
-    <t>2.01</t>
-  </si>
-  <si>
-    <t>Caixa Líquido das Atividades Operacionais</t>
-  </si>
-  <si>
-    <t>1.98</t>
-  </si>
-  <si>
-    <t>Outras Despesas Operacionais</t>
-  </si>
-  <si>
-    <t>1.11</t>
-  </si>
-  <si>
-    <t>Impostos e Contribuições sobre Receita</t>
-  </si>
-  <si>
-    <t>1.10</t>
-  </si>
-  <si>
-    <t>Despesas Administrativas Gerais</t>
-  </si>
-  <si>
-    <t>1.09</t>
-  </si>
-  <si>
-    <t>Despesas Comerciais e de Marketing</t>
-  </si>
-  <si>
-    <t>1.08</t>
-  </si>
-  <si>
-    <t>Pagamentos de Salários e Encargos</t>
-  </si>
-  <si>
-    <t>1.07</t>
-  </si>
-  <si>
-    <t>Pagamentos a Empreiteiros/Subempreiteiros</t>
-  </si>
-  <si>
-    <t>1.06</t>
-  </si>
-  <si>
-    <t>Pagamentos a Fornecedores (Materiais de Construção)</t>
-  </si>
-  <si>
-    <t>1.05</t>
-  </si>
-  <si>
-    <t>Subtotal Entradas Operacionais</t>
-  </si>
-  <si>
-    <t>1.99</t>
-  </si>
-  <si>
-    <t>Outras Receitas Operacionais</t>
-  </si>
-  <si>
-    <t>1.04</t>
-  </si>
-  <si>
-    <t>Recebimentos de Serviços (Taxas de Administração / Corretagem)</t>
-  </si>
-  <si>
-    <t>1.03</t>
-  </si>
-  <si>
-    <t>Recebimentos de Aluguéis</t>
-  </si>
-  <si>
-    <t>1.02</t>
-  </si>
-  <si>
-    <t>Recebimentos de Vendas de Unidades Imobiliárias</t>
-  </si>
-  <si>
-    <t>1.01</t>
-  </si>
-  <si>
-    <t>Total</t>
-  </si>
-  <si>
-    <t>Dez</t>
-  </si>
-  <si>
-    <t>Nov</t>
-  </si>
-  <si>
-    <t>Out</t>
-  </si>
-  <si>
-    <t>Set</t>
-  </si>
-  <si>
-    <t>Ago</t>
-  </si>
-  <si>
-    <t>Jul</t>
-  </si>
-  <si>
-    <t>Jun</t>
-  </si>
-  <si>
-    <t>Mai</t>
-  </si>
-  <si>
-    <t>Abr</t>
-  </si>
-  <si>
-    <t>Mar</t>
-  </si>
-  <si>
-    <t>Fev</t>
-  </si>
-  <si>
-    <t>Jan</t>
-  </si>
-  <si>
-    <t>10. Proteja células de fórmulas para evitar alterações não intencionais.</t>
-  </si>
-  <si>
-    <t>9. Ajuste o mapeamento de contas conforme o plano de contas interno da Ampla.</t>
-  </si>
-  <si>
-    <t>8. Utilize referências absolutas nas fórmulas para manter a consistência ao copiar para novos períodos.</t>
-  </si>
-  <si>
-    <t>7. A variação líquida de caixa (4.01) deve ser a soma dos fluxos líquidos das três atividades.</t>
-  </si>
-  <si>
-    <t>6. Utilize as linhas de subtotal (1.99, 2.98, 3.98) para calcular automaticamente os fluxos líquidos por atividade.</t>
-  </si>
-  <si>
-    <t>5. Registre impostos sobre receita quando da saída de caixa, não pelo fato gerador contábil.</t>
-  </si>
-  <si>
-    <t>4. Detalhe pagamentos a fornecedores por grandes classes de custo (materiais, empreiteiros, etc.).</t>
-  </si>
-  <si>
-    <t>3. Agrupe os recebimentos de clientes por tipo de contrato (vendas, aluguéis, serviços).</t>
-  </si>
-  <si>
-    <t>2. Lance as entradas brutas de caixa separadamente das saídas para cada categoria.</t>
-  </si>
-  <si>
-    <t>1. Utilize apenas valores relacionados a movimentações de caixa efetivas (exclua receitas e despesas a prazo).</t>
-  </si>
-  <si>
-    <t>Orientações para preenchimento da Demonstração do Fluxo de Caixa (Método Direto):</t>
-  </si>
-  <si>
-    <t>Instruções</t>
+    <t>Empresa</t>
+  </si>
+  <si>
+    <t>Banco</t>
+  </si>
+  <si>
+    <t>Conta</t>
+  </si>
+  <si>
+    <t>Se (nos extratos)</t>
+  </si>
+  <si>
+    <t>Então (no DFC)</t>
+  </si>
+  <si>
+    <t>Todas</t>
+  </si>
+  <si>
+    <t>Todos</t>
+  </si>
+  <si>
+    <t>Empresas</t>
+  </si>
+  <si>
+    <t>Bancos</t>
+  </si>
+  <si>
+    <t>Contas</t>
+  </si>
+  <si>
+    <t>DFC</t>
+  </si>
+  <si>
+    <t>PAG AGUA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -481,14 +268,22 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -525,8 +320,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.749992370372631"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -534,26 +341,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -595,14 +387,41 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.749992370372631"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="3" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -613,6 +432,112 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Gráfico 4" descr="Seta para Direita com preenchimento sólido">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B607001B-D30F-4CCC-A4E6-DEE82BEEF1CC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId2"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4210050" y="0"/>
+          <a:ext cx="609600" cy="685800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Variáveis"/>
+      <sheetName val="Arquivos"/>
+      <sheetName val="Relatórios"/>
+      <sheetName val="Empreend.-Filial-Empresa"/>
+      <sheetName val="Contas"/>
+      <sheetName val="Contas-IK"/>
+      <sheetName val="CEF"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AD63709-306E-47D7-A314-DBAC99B4F85D}" name="Tabela1" displayName="Tabela1" ref="F2:F3" totalsRowShown="0" headerRowDxfId="1">
+  <autoFilter ref="F2:F3" xr:uid="{1AD63709-306E-47D7-A314-DBAC99B4F85D}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{E11DE80B-D1AC-4E0F-8514-2B54C784C7A7}" name="Descrição"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A4644A32-86DF-4680-A406-4B53C94BFE14}" name="Tabela2" displayName="Tabela2" ref="A2:D3" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A2:D3" xr:uid="{A4644A32-86DF-4680-A406-4B53C94BFE14}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{09747F26-7800-4998-9D65-D29FA38902A8}" name="Empresa"/>
+    <tableColumn id="2" xr3:uid="{E2813DE1-C567-4EB1-929D-1AB0349AD140}" name="Banco"/>
+    <tableColumn id="3" xr3:uid="{C6C708C1-EA14-416C-BBB8-EF029BDA3E1F}" name="Conta"/>
+    <tableColumn id="4" xr3:uid="{D20D5B7D-D231-4477-B816-34758A2EF602}" name="Descrição"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1402,406 +1327,581 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CD193604-E5F7-47BD-A69A-5284F7B133D5}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FCDBFD3-E4D2-476B-B25F-441255FD953F}">
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="10.85546875" customWidth="1"/>
+    <col min="4" max="4" width="35.7109375" customWidth="1"/>
+    <col min="6" max="6" width="35.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="A1" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" s="16"/>
+      <c r="C1" s="16"/>
+      <c r="D1" s="16"/>
+      <c r="F1" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="H1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="18" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="2">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="3">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4FF4ED5F-8031-4733-9B50-EFDEDEAAEB10}">
+          <x14:formula1>
+            <xm:f>Configurações!$A$2:$A$26</xm:f>
+          </x14:formula1>
+          <xm:sqref>A3</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{250A0206-946F-4E3B-A1FC-3383CEA30FA3}">
+          <x14:formula1>
+            <xm:f>Configurações!$C$2:$C$8</xm:f>
+          </x14:formula1>
+          <xm:sqref>B3</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{80D77F89-4FF3-44EC-B2BA-6BD51B67A140}">
+          <x14:formula1>
+            <xm:f>Configurações!$E$2:$E$66</xm:f>
+          </x14:formula1>
+          <xm:sqref>C3</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AC6E963-55A4-4016-BD3B-C5BBBBA954E5}">
+  <dimension ref="A1:G68"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="3.7109375" customWidth="1"/>
+    <col min="4" max="4" width="3.7109375" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.7109375" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1" s="20" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E2" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="str" cm="1">
+        <f t="array" ref="A3:A26">_xlfn._xlws.SORT(_xlfn.UNIQUE([1]!contas[Empresa]))</f>
+        <v>AMP</v>
+      </c>
+      <c r="C3" t="str" cm="1">
+        <f t="array" ref="C3:C8">_xlfn.UNIQUE(_xlfn._xlws.SORT([1]!contas[Banco]))</f>
+        <v>ABC</v>
+      </c>
+      <c r="E3" t="str" cm="1">
+        <f t="array" ref="E3:E66">_xlfn.LET(_xlpm.bruto, _xlfn.VSTACK([1]!contas[CC (antigo)], [1]!contas[CC (atual)]),
+_xlpm.limpo, _xlfn._xlws.FILTER(_xlpm.bruto, (_xlpm.bruto&lt;&gt;"0") * (_xlpm.bruto&lt;&gt;"-") * (_xlpm.bruto&lt;&gt;"")),
+_xlfn.UNIQUE(TEXT(_xlfn._xlws.SORT(_xlpm.limpo), "@")))</f>
+        <v>3701</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <v>AVR</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CEF</v>
+      </c>
+      <c r="E4" s="21" t="str">
+        <v>002292447-9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <v>AVS</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Itaú</v>
+      </c>
+      <c r="E5" s="21" t="str">
+        <v>002292448-7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <v>BUT</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Linkpay</v>
+      </c>
+      <c r="E6" s="21" t="str">
+        <v>03852-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <v>CBL</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Paulista</v>
+      </c>
+      <c r="E7" s="21" t="str">
+        <v>06340-0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <v>CHR</v>
+      </c>
+      <c r="C8" t="str">
+        <v>QI Tech</v>
+      </c>
+      <c r="E8" s="21" t="str">
+        <v>09700-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <v>CPE</v>
+      </c>
+      <c r="E9" s="21" t="str">
+        <v>2245-8</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="str">
+        <v>DEC</v>
+      </c>
+      <c r="E10" s="21" t="str">
+        <v>2278-4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="str">
+        <v>DPF</v>
+      </c>
+      <c r="E11" s="21" t="str">
+        <v>2362-4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="str">
+        <v>ENC</v>
+      </c>
+      <c r="E12" s="21" t="str">
+        <v>2399-3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="str">
+        <v>GRA</v>
+      </c>
+      <c r="E13" s="21" t="str">
+        <v>2419-1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" t="str">
+        <v>INC</v>
+      </c>
+      <c r="E14" s="21" t="str">
+        <v>2420-5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" t="str">
+        <v>JRP</v>
+      </c>
+      <c r="E15" s="21" t="str">
+        <v>2429-9</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" t="str">
+        <v>JSP</v>
+      </c>
+      <c r="E16" s="21" t="str">
+        <v>2480-9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" t="str">
+        <v>LCG</v>
+      </c>
+      <c r="E17" s="21" t="str">
+        <v>2498-1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18" t="str">
+        <v>LUC</v>
+      </c>
+      <c r="E18" s="21" t="str">
+        <v>2505-8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="str">
+        <v>PDI</v>
+      </c>
+      <c r="E19" s="21" t="str">
+        <v>29548-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="str">
+        <v>POM</v>
+      </c>
+      <c r="E20" s="21" t="str">
+        <v>29757-4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="str">
+        <v>SAU</v>
+      </c>
+      <c r="E21" s="21" t="str">
+        <v>3455-6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" t="str">
+        <v>SBB</v>
+      </c>
+      <c r="E22" s="21" t="str">
+        <v>576265461-0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" t="str">
+        <v>SN2</v>
+      </c>
+      <c r="E23" s="21" t="str">
+        <v>576268473-0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A24" t="str">
+        <v>SN4</v>
+      </c>
+      <c r="E24" s="21" t="str">
+        <v>576533068-8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="str">
+        <v>SOC</v>
+      </c>
+      <c r="E25" s="21" t="str">
+        <v>577141188-0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="str">
+        <v>USL</v>
+      </c>
+      <c r="E26" s="21" t="str">
+        <v>577180827-6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E27" s="21" t="str">
+        <v>577180924-8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E28" s="21" t="str">
+        <v>577181031-9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E29" s="21" t="str">
+        <v>577243227-0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E30" s="21" t="str">
+        <v>577243229-6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E31" s="21" t="str">
+        <v>577243231-8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E32" s="21" t="str">
+        <v>577294854-3</v>
+      </c>
+    </row>
+    <row r="33" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E33" s="21" t="str">
+        <v>577294862-4</v>
+      </c>
+    </row>
+    <row r="34" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E34" s="21" t="str">
+        <v>577565836-8</v>
+      </c>
+    </row>
+    <row r="35" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E35" s="21" t="str">
+        <v>578129123-3</v>
+      </c>
+    </row>
+    <row r="36" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E36" s="21" t="str">
+        <v>578317306-8</v>
+      </c>
+    </row>
+    <row r="37" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E37" s="21" t="str">
+        <v>579133302-8</v>
+      </c>
+    </row>
+    <row r="38" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E38" s="21" t="str">
+        <v>579133317-6</v>
+      </c>
+    </row>
+    <row r="39" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E39" s="21" t="str">
+        <v>579133324-9</v>
+      </c>
+    </row>
+    <row r="40" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E40" s="21" t="str">
+        <v>579133332-0</v>
+      </c>
+    </row>
+    <row r="41" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E41" s="21" t="str">
+        <v>579133363-0</v>
+      </c>
+    </row>
+    <row r="42" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E42" s="21" t="str">
+        <v>579133369-9</v>
+      </c>
+    </row>
+    <row r="43" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E43" s="21" t="str">
+        <v>579897189-5</v>
+      </c>
+    </row>
+    <row r="44" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E44" s="21" t="str">
+        <v>586376394-5</v>
+      </c>
+    </row>
+    <row r="45" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E45" s="21" t="str">
+        <v>586376423-2</v>
+      </c>
+    </row>
+    <row r="46" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E46" s="21" t="str">
+        <v>600-0</v>
+      </c>
+    </row>
+    <row r="47" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E47" s="21" t="str">
+        <v>659-0</v>
+      </c>
+    </row>
+    <row r="48" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E48" s="21" t="str">
+        <v>742397833-8</v>
+      </c>
+    </row>
+    <row r="49" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E49" s="21" t="str">
+        <v>793-7</v>
+      </c>
+    </row>
+    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E50" s="21" t="str">
+        <v>7986045-7</v>
+      </c>
+    </row>
+    <row r="51" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E51" s="21" t="str">
+        <v>97588-9</v>
+      </c>
+    </row>
+    <row r="52" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E52" s="21" t="str">
+        <v>97589-7</v>
+      </c>
+    </row>
+    <row r="53" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E53" s="21" t="str">
+        <v>97648-1</v>
+      </c>
+    </row>
+    <row r="54" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E54" s="21" t="str">
+        <v>98426-1</v>
+      </c>
+    </row>
+    <row r="55" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E55" s="21" t="str">
+        <v>99267-3</v>
+      </c>
+    </row>
+    <row r="56" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E56" s="21" t="str">
+        <v>99310-1</v>
+      </c>
+    </row>
+    <row r="57" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E57" s="21" t="str">
+        <v>99651-8</v>
+      </c>
+    </row>
+    <row r="58" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E58" s="21" t="str">
+        <v>99653-4</v>
+      </c>
+    </row>
+    <row r="59" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E59" s="21" t="str">
+        <v>99660-9</v>
+      </c>
+    </row>
+    <row r="60" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E60" s="21" t="str">
+        <v>99664-1</v>
+      </c>
+    </row>
+    <row r="61" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E61" s="21" t="str">
+        <v>99681-5</v>
+      </c>
+    </row>
+    <row r="62" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E62" s="21" t="str">
+        <v>99715-1</v>
+      </c>
+    </row>
+    <row r="63" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E63" s="21" t="str">
+        <v>99716-9</v>
+      </c>
+    </row>
+    <row r="64" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E64" s="21" t="str">
+        <v>99725-0</v>
+      </c>
+    </row>
+    <row r="65" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E65" s="21" t="str">
+        <v>99756-5</v>
+      </c>
+    </row>
+    <row r="66" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E66" s="21" t="str">
+        <v>99853-0</v>
+      </c>
+    </row>
+    <row r="67" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E67" s="21"/>
+    </row>
+    <row r="68" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E68" s="21"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DE0B94E-0419-42F5-8555-F770A44E2D08}">
-  <dimension ref="A1:O34"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="15" t="s">
-        <v>124</v>
-      </c>
-      <c r="D1" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="E1" s="15" t="s">
-        <v>122</v>
-      </c>
-      <c r="F1" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="G1" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="H1" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="I1" s="15" t="s">
-        <v>118</v>
-      </c>
-      <c r="J1" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="K1" s="15" t="s">
-        <v>116</v>
-      </c>
-      <c r="L1" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="M1" s="15" t="s">
-        <v>114</v>
-      </c>
-      <c r="N1" s="15" t="s">
-        <v>113</v>
-      </c>
-      <c r="O1" s="15" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>111</v>
-      </c>
-      <c r="B2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>109</v>
-      </c>
-      <c r="B3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>105</v>
-      </c>
-      <c r="B5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>103</v>
-      </c>
-      <c r="B6" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>101</v>
-      </c>
-      <c r="B7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>99</v>
-      </c>
-      <c r="B8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>97</v>
-      </c>
-      <c r="B9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>95</v>
-      </c>
-      <c r="B10" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>93</v>
-      </c>
-      <c r="B11" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>91</v>
-      </c>
-      <c r="B12" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>89</v>
-      </c>
-      <c r="B13" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>87</v>
-      </c>
-      <c r="B14" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>85</v>
-      </c>
-      <c r="B15" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>83</v>
-      </c>
-      <c r="B16" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>81</v>
-      </c>
-      <c r="B17" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>79</v>
-      </c>
-      <c r="B18" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>77</v>
-      </c>
-      <c r="B19" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>75</v>
-      </c>
-      <c r="B20" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>73</v>
-      </c>
-      <c r="B21" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>71</v>
-      </c>
-      <c r="B22" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>69</v>
-      </c>
-      <c r="B23" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>67</v>
-      </c>
-      <c r="B24" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>65</v>
-      </c>
-      <c r="B25" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>63</v>
-      </c>
-      <c r="B26" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>61</v>
-      </c>
-      <c r="B27" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>59</v>
-      </c>
-      <c r="B28" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>57</v>
-      </c>
-      <c r="B29" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>55</v>
-      </c>
-      <c r="B30" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>53</v>
-      </c>
-      <c r="B31" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>51</v>
-      </c>
-      <c r="B32" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>49</v>
-      </c>
-      <c r="B33" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>47</v>
-      </c>
-      <c r="B34" t="s">
-        <v>46</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EA864A3-80F6-45EA-B46F-4714BF885D6B}">
-  <dimension ref="A1:A12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>125</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
     <xsd:import namespace="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
@@ -1996,27 +2096,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7BFC80B-7A55-4801-9844-CCCBA392669F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7E4AD77-7BCF-4163-8EFB-17D24A162300}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5F1B5B1-5FBC-42BF-93E0-A1561CA25062}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2033,23 +2132,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7E4AD77-7BCF-4163-8EFB-17D24A162300}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
-    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7BFC80B-7A55-4801-9844-CCCBA392669F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Enhance e_extratos function to support Excel file generation with multiple sheets; add new template and data files; remove outdated empreendimentos.xlsx.
</commit_message>
<xml_diff>
--- a/templates/Template-DFC.xlsx
+++ b/templates/Template-DFC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="400" documentId="8_{482EB0F2-8EC4-40C5-8B55-F33B1732A6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{56DE95E9-BB3E-41E9-BF20-7F01584FABD5}"/>
+  <xr:revisionPtr revIDLastSave="416" documentId="8_{482EB0F2-8EC4-40C5-8B55-F33B1732A6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BAF1A6D-C0A2-4B28-82DE-5F7AA8F567A7}"/>
   <bookViews>
-    <workbookView xWindow="-43200" yWindow="4245" windowWidth="14400" windowHeight="7800" activeTab="2" xr2:uid="{E8652140-B299-493A-AAA8-27682F0F7EF9}"/>
+    <workbookView xWindow="-28920" yWindow="-1305" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{E8652140-B299-493A-AAA8-27682F0F7EF9}"/>
   </bookViews>
   <sheets>
     <sheet name="DFC" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <externalReferences>
     <externalReference r:id="rId4"/>
   </externalReferences>
-  <calcPr calcId="191029" calcCompleted="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="59">
   <si>
     <t>Código</t>
   </si>
@@ -236,14 +236,17 @@
     <t>DFC</t>
   </si>
   <si>
-    <t>PAG AGUA</t>
+    <t>Descrição nos extratos</t>
+  </si>
+  <si>
+    <t>Descrição no DFC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -278,6 +281,12 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -402,21 +411,12 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="3" tint="0.749992370372631"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="3" tint="0.499984740745262"/>
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -438,23 +438,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>609599</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>161925</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>9524</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Gráfico 4" descr="Seta para Direita com preenchimento sólido">
+        <xdr:cNvPr id="3" name="Gráfico 2" descr="Seta para Direita com preenchimento sólido">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B607001B-D30F-4CCC-A4E6-DEE82BEEF1CC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4CD96445-36FC-4103-8EB8-F1932AFD13E7}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -476,8 +476,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4210050" y="0"/>
-          <a:ext cx="609600" cy="685800"/>
+          <a:off x="1943099" y="0"/>
+          <a:ext cx="3057525" cy="333375"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -503,38 +503,31 @@
       <sheetName val="Contas"/>
       <sheetName val="Contas-IK"/>
       <sheetName val="CEF"/>
+      <sheetName val="Mapeamento dos dados"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
+      <sheetData sheetId="0" refreshError="1"/>
+      <sheetData sheetId="1" refreshError="1"/>
+      <sheetData sheetId="2" refreshError="1"/>
+      <sheetData sheetId="3" refreshError="1"/>
       <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
+      <sheetData sheetId="5" refreshError="1"/>
+      <sheetData sheetId="6" refreshError="1"/>
+      <sheetData sheetId="7" refreshError="1"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1AD63709-306E-47D7-A314-DBAC99B4F85D}" name="Tabela1" displayName="Tabela1" ref="F2:F3" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="F2:F3" xr:uid="{1AD63709-306E-47D7-A314-DBAC99B4F85D}"/>
-  <tableColumns count="1">
-    <tableColumn id="1" xr3:uid="{E11DE80B-D1AC-4E0F-8514-2B54C784C7A7}" name="Descrição"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A4644A32-86DF-4680-A406-4B53C94BFE14}" name="Tabela2" displayName="Tabela2" ref="A2:D3" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A2:D3" xr:uid="{A4644A32-86DF-4680-A406-4B53C94BFE14}"/>
-  <tableColumns count="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A4644A32-86DF-4680-A406-4B53C94BFE14}" name="Tabela2" displayName="Tabela2" ref="A2:E3" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A2:E3" xr:uid="{A4644A32-86DF-4680-A406-4B53C94BFE14}"/>
+  <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{09747F26-7800-4998-9D65-D29FA38902A8}" name="Empresa"/>
     <tableColumn id="2" xr3:uid="{E2813DE1-C567-4EB1-929D-1AB0349AD140}" name="Banco"/>
     <tableColumn id="3" xr3:uid="{C6C708C1-EA14-416C-BBB8-EF029BDA3E1F}" name="Conta"/>
-    <tableColumn id="4" xr3:uid="{D20D5B7D-D231-4477-B816-34758A2EF602}" name="Descrição"/>
+    <tableColumn id="6" xr3:uid="{467D06F7-18B0-4033-87AD-6DDE247DBEE4}" name="Descrição nos extratos"/>
+    <tableColumn id="4" xr3:uid="{D20D5B7D-D231-4477-B816-34758A2EF602}" name="Descrição no DFC"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1328,29 +1321,28 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FCDBFD3-E4D2-476B-B25F-441255FD953F}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
-    <col min="4" max="4" width="35.7109375" customWidth="1"/>
-    <col min="6" max="6" width="35.7109375" customWidth="1"/>
+    <col min="4" max="5" width="45.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="26.25" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:7" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A1" s="15" t="s">
         <v>49</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
       <c r="D1" s="16"/>
-      <c r="F1" s="17" t="s">
+      <c r="E1" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="H1" t="s">
+      <c r="G1" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="19" t="s">
         <v>46</v>
       </c>
@@ -1361,35 +1353,21 @@
         <v>48</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="18" t="s">
-        <v>1</v>
-      </c>
-      <c r="H2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="G2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C3" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" t="s">
-        <v>57</v>
-      </c>
-    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>
-  <tableParts count="2">
+  <tableParts count="1">
     <tablePart r:id="rId2"/>
-    <tablePart r:id="rId3"/>
   </tableParts>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -1410,7 +1388,7 @@
           <x14:formula1>
             <xm:f>Configurações!$E$2:$E$66</xm:f>
           </x14:formula1>
-          <xm:sqref>C3</xm:sqref>
+          <xm:sqref>C3:D3</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1882,26 +1860,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
     <xsd:import namespace="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
@@ -2096,10 +2054,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7BFC80B-7A55-4801-9844-CCCBA392669F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5F1B5B1-5FBC-42BF-93E0-A1561CA25062}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2116,20 +2105,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5F1B5B1-5FBC-42BF-93E0-A1561CA25062}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7BFC80B-7A55-4801-9844-CCCBA392669F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
-    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add CMF data extraction to e_extratos and enhance gerar_xlsx for template handling
</commit_message>
<xml_diff>
--- a/templates/Template-DFC.xlsx
+++ b/templates/Template-DFC.xlsx
@@ -1,24 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://incorporadoraampla.sharepoint.com/sites/Controladoria/Documentos Compartilhados/amplaGitHub/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="416" documentId="8_{482EB0F2-8EC4-40C5-8B55-F33B1732A6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BAF1A6D-C0A2-4B28-82DE-5F7AA8F567A7}"/>
+  <xr:revisionPtr revIDLastSave="447" documentId="8_{482EB0F2-8EC4-40C5-8B55-F33B1732A6B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{462043C4-ACE6-46FA-AE91-25783254407F}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-1305" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{E8652140-B299-493A-AAA8-27682F0F7EF9}"/>
+    <workbookView xWindow="20370" yWindow="-8025" windowWidth="29040" windowHeight="15840" tabRatio="677" activeTab="6" xr2:uid="{E8652140-B299-493A-AAA8-27682F0F7EF9}"/>
   </bookViews>
   <sheets>
-    <sheet name="DFC" sheetId="1" r:id="rId1"/>
-    <sheet name="Mapeamento" sheetId="5" r:id="rId2"/>
-    <sheet name="Configurações" sheetId="6" r:id="rId3"/>
+    <sheet name="Extratos" sheetId="7" r:id="rId1"/>
+    <sheet name="Resumo - Lançamentos" sheetId="9" r:id="rId2"/>
+    <sheet name="Extratos - Ik" sheetId="8" r:id="rId3"/>
+    <sheet name="Contas mensal" sheetId="10" r:id="rId4"/>
+    <sheet name="Empresas mensal" sheetId="11" r:id="rId5"/>
+    <sheet name="DFC" sheetId="1" r:id="rId6"/>
+    <sheet name="Mapeamento" sheetId="5" r:id="rId7"/>
+    <sheet name="Configurações" sheetId="6" r:id="rId8"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId4"/>
+    <externalReference r:id="rId9"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -501,19 +506,19 @@
       <sheetName val="Relatórios"/>
       <sheetName val="Empreend.-Filial-Empresa"/>
       <sheetName val="Contas"/>
+      <sheetName val="Contas_A"/>
       <sheetName val="Contas-IK"/>
       <sheetName val="CEF"/>
-      <sheetName val="Mapeamento dos dados"/>
     </sheetNames>
     <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1" refreshError="1"/>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
       <sheetData sheetId="4"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -849,7 +854,70 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3D1D357-3BE0-4DC5-9E1D-DD9B9CF83E4C}">
+  <sheetPr>
+    <tabColor theme="3" tint="0.499984740745262"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2FABB518-66AE-4125-A185-69F12DB2F4AC}">
+  <sheetPr>
+    <tabColor theme="3" tint="0.499984740745262"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{17C21122-7C7A-407C-AC37-AA0B6EA5FB6A}">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEB2E33D-BE12-4612-BFFD-1FDAF9485537}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8ADFF572-910F-47DA-93FB-6B8842E04057}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A93FF019-ACA5-4674-AAA1-FFC1EFB894DF}">
+  <sheetPr>
+    <tabColor theme="6" tint="0.39997558519241921"/>
+  </sheetPr>
   <dimension ref="A1:F35"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="2" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1319,8 +1387,11 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FCDBFD3-E4D2-476B-B25F-441255FD953F}">
+  <sheetPr>
+    <tabColor theme="0" tint="-0.249977111117893"/>
+  </sheetPr>
   <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1396,8 +1467,11 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7AC6E963-55A4-4016-BD3B-C5BBBBA954E5}">
+  <sheetPr>
+    <tabColor theme="0" tint="-0.249977111117893"/>
+  </sheetPr>
   <dimension ref="A1:G68"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1860,6 +1934,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101006C56FB2846673243A9735D5EC6051572" ma:contentTypeVersion="11" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="36569ac63cfce8ff0f8884bc80e67f1c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5a5f483f-f768-438e-b4ef-63f46a7558dd" xmlns:ns3="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2040da04b75a9ea4fe796fa8180f8ca6" ns2:_="" ns3:_="">
     <xsd:import namespace="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
@@ -2054,17 +2139,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5a5f483f-f768-438e-b4ef-63f46a7558dd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="dd8c73df-45bd-468c-aae5-f3faedcbd5e2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2075,6 +2149,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7E4AD77-7BCF-4163-8EFB-17D24A162300}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
+    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A5F1B5B1-5FBC-42BF-93E0-A1561CA25062}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2093,17 +2178,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7E4AD77-7BCF-4163-8EFB-17D24A162300}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="5a5f483f-f768-438e-b4ef-63f46a7558dd"/>
-    <ds:schemaRef ds:uri="dd8c73df-45bd-468c-aae5-f3faedcbd5e2"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E7BFC80B-7A55-4801-9844-CCCBA392669F}">
   <ds:schemaRefs>

</xml_diff>